<commit_message>
Kestrel part 1: make the planted duplicate a true duplicate
The planted duplicate bill had the same invoice number as Moraine's March
bill but a different amount, so it was not a duplicate in fact (the new
duplicate-bill check correctly called it 'different amounts'). The original
March invoice is now 18,432.50 as well; the difference moves to Moraine's
April bill and purchase order, so every total (purchases, bills, payments,
POs, AP) is unchanged. Key updated; frozen part-0 key still 13/13.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/case-studies/kestrel-valley-cycle/data/quickbooks/Journal.xlsx
+++ b/case-studies/kestrel-valley-cycle/data/quickbooks/Journal.xlsx
@@ -20560,7 +20560,7 @@
         </is>
       </c>
       <c r="H981" s="1" t="n">
-        <v>169202.82</v>
+        <v>18432.5</v>
       </c>
       <c r="J981" t="inlineStr">
         <is>
@@ -20585,15 +20585,15 @@
         </is>
       </c>
       <c r="I982" s="1" t="n">
-        <v>169202.82</v>
+        <v>18432.5</v>
       </c>
     </row>
     <row r="983">
       <c r="H983" s="1" t="n">
-        <v>169202.82</v>
+        <v>18432.5</v>
       </c>
       <c r="I983" s="1" t="n">
-        <v>169202.82</v>
+        <v>18432.5</v>
       </c>
     </row>
     <row r="984">
@@ -23229,7 +23229,7 @@
         </is>
       </c>
       <c r="H1111" s="1" t="n">
-        <v>203043.39</v>
+        <v>353813.71</v>
       </c>
       <c r="J1111" t="inlineStr">
         <is>
@@ -23254,15 +23254,15 @@
         </is>
       </c>
       <c r="I1112" s="1" t="n">
-        <v>203043.39</v>
+        <v>353813.71</v>
       </c>
     </row>
     <row r="1113">
       <c r="H1113" s="1" t="n">
-        <v>203043.39</v>
+        <v>353813.71</v>
       </c>
       <c r="I1113" s="1" t="n">
-        <v>203043.39</v>
+        <v>353813.71</v>
       </c>
     </row>
     <row r="1114">

</xml_diff>